<commit_message>
Adiciona previa segura da importacao de cursistas
</commit_message>
<xml_diff>
--- a/frontend/public/modelos/modelo-importacao-cursistas.xlsx
+++ b/frontend/public/modelos/modelo-importacao-cursistas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rayll\Desktop\Transforma Educação PB\transforma\frontend\public\modelos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AED77ECB-8E8B-448E-B130-2B84EE4B37EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4528D8A7-7AB6-4F15-B2DD-9310631A0CAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3384" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{018811C3-D330-4AC2-90E4-ADE8255937C8}"/>
   </bookViews>
@@ -18,8 +18,8 @@
     <sheet name="INSTRUCOES" sheetId="1" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">PERFIL_DOCENTE!$A$1:$Y$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">USUARIOS!$A$1:$E$1</definedName>
+    <definedName name="_FilterDatabase" localSheetId="1" hidden="1">PERFIL_DOCENTE!$A$1:$Y$1</definedName>
+    <definedName name="_FilterDatabase" localSheetId="0" hidden="1">USUARIOS!$A$1:$E$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="50">
   <si>
     <t>CPF</t>
   </si>
@@ -165,15 +165,9 @@
     <t>CPF ja cadastrado</t>
   </si>
   <si>
-    <t>O sistema atualiza o cadastro existente. Nao cria uma segunda pessoa com o mesmo CPF.</t>
-  </si>
-  <si>
     <t>CPF novo</t>
   </si>
   <si>
-    <t>Se for valido e ainda nao existir, o sistema adiciona o cursista a lista.</t>
-  </si>
-  <si>
     <t>Duplicado no arquivo</t>
   </si>
   <si>
@@ -184,6 +178,18 @@
   </si>
   <si>
     <t>Nao altere os nomes das abas USUARIOS e PERFIL_DOCENTE nem os cabecalhos das colunas.</t>
+  </si>
+  <si>
+    <t>O sistema mostra o registro como duplicado e nao altera seus dados, senha ou inscricoes.</t>
+  </si>
+  <si>
+    <t>Se for valido e ainda nao existir, aparece na previa e so entra na lista depois da confirmacao.</t>
+  </si>
+  <si>
+    <t>Conferencia antes de gravar</t>
+  </si>
+  <si>
+    <t>O envio primeiro valida a planilha. Revise os novos e baixe os invalidos e duplicados antes de confirmar.</t>
   </si>
 </sst>
 </file>
@@ -279,13 +285,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -293,6 +293,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -751,7 +757,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D44AFF95-45F4-4110-8D7B-85FE77605684}">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="13.2"/>
   <cols>
     <col min="1" max="1" width="24.77734375" style="2" customWidth="1"/>
@@ -761,130 +767,136 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="34.049999999999997" customHeight="1">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
     </row>
     <row r="3" spans="1:4" ht="34.049999999999997" customHeight="1">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
+      <c r="C3" s="8"/>
+      <c r="D3" s="8"/>
     </row>
     <row r="4" spans="1:4" ht="34.049999999999997" customHeight="1">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="C4" s="9"/>
-      <c r="D4" s="9"/>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
     </row>
     <row r="5" spans="1:4" ht="34.049999999999997" customHeight="1">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
     </row>
     <row r="6" spans="1:4" ht="34.049999999999997" customHeight="1">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
     </row>
     <row r="7" spans="1:4" ht="34.049999999999997" customHeight="1">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
     </row>
     <row r="8" spans="1:4" ht="34.049999999999997" customHeight="1">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="7"/>
     </row>
     <row r="9" spans="1:4" ht="34.049999999999997" customHeight="1">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
     </row>
     <row r="10" spans="1:4" ht="34.049999999999997" customHeight="1">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="B10" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+    </row>
+    <row r="11" spans="1:4" ht="34.049999999999997" customHeight="1">
+      <c r="A11" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="C10" s="9"/>
-      <c r="D10" s="9"/>
-    </row>
-    <row r="11" spans="1:4" ht="34.049999999999997" customHeight="1">
-      <c r="A11" s="6" t="s">
+      <c r="B11" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C11" s="8"/>
+      <c r="D11" s="8"/>
+    </row>
+    <row r="12" spans="1:4" ht="34.049999999999997" customHeight="1">
+      <c r="A12" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B12" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-    </row>
-    <row r="12" spans="1:4" ht="34.049999999999997" customHeight="1">
-      <c r="A12" s="8" t="s">
+      <c r="C12" s="7"/>
+      <c r="D12" s="7"/>
+    </row>
+    <row r="13" spans="1:4" ht="34.049999999999997" customHeight="1">
+      <c r="A13" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="B13" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
-    </row>
-    <row r="13" spans="1:4" ht="34.049999999999997" customHeight="1">
-      <c r="A13" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="B13" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="8"/>
+    </row>
+    <row r="14" spans="1:4" ht="34.049999999999997" customHeight="1">
+      <c r="A14" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C14" s="7"/>
+      <c r="D14" s="7"/>
     </row>
   </sheetData>
-  <mergeCells count="12">
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="B12:D12"/>
+  <mergeCells count="13">
+    <mergeCell ref="B14:D14"/>
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="B3:D3"/>
@@ -892,7 +904,13 @@
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="B6:D6"/>
     <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="B12:D12"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>